<commit_message>
Integra os 16 inimigos das florestas iniciais
Adiciona PNGs transparentes, animações e impactos por monstro, chefes solo com escala 1,25 e atributos derivados das fichas iniciais. Amplia a planilha para 79 perfis e preserva as demais regiões e a atualização de conquistas.

Validado em Godot 4.7.2: cadastro, planilha, combate, rotas, limites, conquistas e apresentação PC/mobile. APK Android código 23 com assinatura anterior preservada.
</commit_message>
<xml_diff>
--- a/data/inimigos.xlsx
+++ b/data/inimigos.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inimigos" sheetId="1" r:id="R90da68b7ca994f98"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guia" sheetId="2" r:id="Re5624643c4374a99"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inimigos" sheetId="1" r:id="Reee9ab94d962422f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guia" sheetId="2" r:id="R1ca0f8dc0e0640df"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -174,7 +174,7 @@
         <x:color rgb="FFA12525"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDE6E6"/>
         </x:patternFill>
       </x:fill>
@@ -184,8 +184,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="InimigosBalanceamento" displayName="InimigosBalanceamento" ref="A1:M64" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:M64"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="InimigosBalanceamento" displayName="InimigosBalanceamento" ref="A1:M80" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:M80"/>
   <x:tableColumns count="13">
     <x:tableColumn id="1" name="id"/>
     <x:tableColumn id="2" name="tipo"/>
@@ -3042,6 +3042,662 @@
         <x:v>2.9</x:v>
       </x:c>
     </x:row>
+    <x:row r="65">
+      <x:c r="A65" s="3" t="str">
+        <x:v>phase1_winter_wolf</x:v>
+      </x:c>
+      <x:c r="B65" s="3" t="str">
+        <x:v>Comum</x:v>
+      </x:c>
+      <x:c r="C65" s="11" t="str">
+        <x:v>Floresta Inverno</x:v>
+      </x:c>
+      <x:c r="D65" s="4" t="str">
+        <x:v>Lobo Branco</x:v>
+      </x:c>
+      <x:c r="E65" s="3" t="str">
+        <x:v>assassin</x:v>
+      </x:c>
+      <x:c r="F65" s="5" t="n">
+        <x:v>118.70833333333334</x:v>
+      </x:c>
+      <x:c r="G65" s="5" t="n">
+        <x:v>16.8125</x:v>
+      </x:c>
+      <x:c r="H65" s="5" t="n">
+        <x:v>0.6250000000000001</x:v>
+      </x:c>
+      <x:c r="I65" s="5" t="n">
+        <x:v>0.875</x:v>
+      </x:c>
+      <x:c r="J65" s="6" t="n">
+        <x:v>58.33333333333333</x:v>
+      </x:c>
+      <x:c r="K65" s="6" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="L65" s="7" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M65" s="5" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="66">
+      <x:c r="A66" s="3" t="str">
+        <x:v>phase1_winter_owl</x:v>
+      </x:c>
+      <x:c r="B66" s="3" t="str">
+        <x:v>Comum</x:v>
+      </x:c>
+      <x:c r="C66" s="11" t="str">
+        <x:v>Floresta Inverno</x:v>
+      </x:c>
+      <x:c r="D66" s="4" t="str">
+        <x:v>Coruja Branca</x:v>
+      </x:c>
+      <x:c r="E66" s="3" t="str">
+        <x:v>assassin</x:v>
+      </x:c>
+      <x:c r="F66" s="5" t="n">
+        <x:v>97.125</x:v>
+      </x:c>
+      <x:c r="G66" s="5" t="n">
+        <x:v>15.691666666666668</x:v>
+      </x:c>
+      <x:c r="H66" s="5" t="n">
+        <x:v>0.5208333333333334</x:v>
+      </x:c>
+      <x:c r="I66" s="5" t="n">
+        <x:v>0.7291666666666665</x:v>
+      </x:c>
+      <x:c r="J66" s="6" t="n">
+        <x:v>58.33333333333333</x:v>
+      </x:c>
+      <x:c r="K66" s="6" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="L66" s="7" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M66" s="5" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="67">
+      <x:c r="A67" s="3" t="str">
+        <x:v>phase1_winter_hunter</x:v>
+      </x:c>
+      <x:c r="B67" s="3" t="str">
+        <x:v>Comum</x:v>
+      </x:c>
+      <x:c r="C67" s="11" t="str">
+        <x:v>Floresta Inverno</x:v>
+      </x:c>
+      <x:c r="D67" s="4" t="str">
+        <x:v>Caçador de Inverno</x:v>
+      </x:c>
+      <x:c r="E67" s="3" t="str">
+        <x:v>ranger</x:v>
+      </x:c>
+      <x:c r="F67" s="5" t="n">
+        <x:v>118.70833333333334</x:v>
+      </x:c>
+      <x:c r="G67" s="5" t="n">
+        <x:v>22.41666666666667</x:v>
+      </x:c>
+      <x:c r="H67" s="5" t="n">
+        <x:v>0.6250000000000001</x:v>
+      </x:c>
+      <x:c r="I67" s="5" t="n">
+        <x:v>0.875</x:v>
+      </x:c>
+      <x:c r="J67" s="6" t="n">
+        <x:v>37.33333333333333</x:v>
+      </x:c>
+      <x:c r="K67" s="6" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="L67" s="7" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M67" s="5" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="68">
+      <x:c r="A68" s="3" t="str">
+        <x:v>phase1_winter_moose</x:v>
+      </x:c>
+      <x:c r="B68" s="3" t="str">
+        <x:v>Chefe</x:v>
+      </x:c>
+      <x:c r="C68" s="11" t="str">
+        <x:v>Floresta Inverno</x:v>
+      </x:c>
+      <x:c r="D68" s="4" t="str">
+        <x:v>Alce</x:v>
+      </x:c>
+      <x:c r="E68" s="3" t="str">
+        <x:v>vanguard</x:v>
+      </x:c>
+      <x:c r="F68" s="5" t="n">
+        <x:v>949.6666666666667</x:v>
+      </x:c>
+      <x:c r="G68" s="5" t="n">
+        <x:v>23.5375</x:v>
+      </x:c>
+      <x:c r="H68" s="5" t="n">
+        <x:v>2.1875000000000004</x:v>
+      </x:c>
+      <x:c r="I68" s="5" t="n">
+        <x:v>3.0625</x:v>
+      </x:c>
+      <x:c r="J68" s="6" t="n">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="K68" s="6" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="L68" s="7" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M68" s="5" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="69">
+      <x:c r="A69" s="3" t="str">
+        <x:v>phase1_autumn_hare</x:v>
+      </x:c>
+      <x:c r="B69" s="3" t="str">
+        <x:v>Comum</x:v>
+      </x:c>
+      <x:c r="C69" s="11" t="str">
+        <x:v>Floresta Outono</x:v>
+      </x:c>
+      <x:c r="D69" s="4" t="str">
+        <x:v>Lebre de Dentes Afiados</x:v>
+      </x:c>
+      <x:c r="E69" s="3" t="str">
+        <x:v>assassin</x:v>
+      </x:c>
+      <x:c r="F69" s="5" t="n">
+        <x:v>75.54166666666667</x:v>
+      </x:c>
+      <x:c r="G69" s="5" t="n">
+        <x:v>12.329166666666667</x:v>
+      </x:c>
+      <x:c r="H69" s="5" t="n">
+        <x:v>0.31250000000000006</x:v>
+      </x:c>
+      <x:c r="I69" s="5" t="n">
+        <x:v>0.4375</x:v>
+      </x:c>
+      <x:c r="J69" s="6" t="n">
+        <x:v>65.33333333333333</x:v>
+      </x:c>
+      <x:c r="K69" s="6" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="L69" s="7" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M69" s="5" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="70">
+      <x:c r="A70" s="3" t="str">
+        <x:v>phase1_autumn_fox</x:v>
+      </x:c>
+      <x:c r="B70" s="3" t="str">
+        <x:v>Comum</x:v>
+      </x:c>
+      <x:c r="C70" s="11" t="str">
+        <x:v>Floresta Outono</x:v>
+      </x:c>
+      <x:c r="D70" s="4" t="str">
+        <x:v>Raposa</x:v>
+      </x:c>
+      <x:c r="E70" s="3" t="str">
+        <x:v>assassin</x:v>
+      </x:c>
+      <x:c r="F70" s="5" t="n">
+        <x:v>97.125</x:v>
+      </x:c>
+      <x:c r="G70" s="5" t="n">
+        <x:v>14.570833333333335</x:v>
+      </x:c>
+      <x:c r="H70" s="5" t="n">
+        <x:v>0.5208333333333334</x:v>
+      </x:c>
+      <x:c r="I70" s="5" t="n">
+        <x:v>0.7291666666666665</x:v>
+      </x:c>
+      <x:c r="J70" s="6" t="n">
+        <x:v>58.33333333333333</x:v>
+      </x:c>
+      <x:c r="K70" s="6" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="L70" s="7" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M70" s="5" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="71">
+      <x:c r="A71" s="3" t="str">
+        <x:v>phase1_autumn_wolf</x:v>
+      </x:c>
+      <x:c r="B71" s="3" t="str">
+        <x:v>Comum</x:v>
+      </x:c>
+      <x:c r="C71" s="11" t="str">
+        <x:v>Floresta Outono</x:v>
+      </x:c>
+      <x:c r="D71" s="4" t="str">
+        <x:v>Lobo Preto</x:v>
+      </x:c>
+      <x:c r="E71" s="3" t="str">
+        <x:v>assassin</x:v>
+      </x:c>
+      <x:c r="F71" s="5" t="n">
+        <x:v>129.5</x:v>
+      </x:c>
+      <x:c r="G71" s="5" t="n">
+        <x:v>19.054166666666667</x:v>
+      </x:c>
+      <x:c r="H71" s="5" t="n">
+        <x:v>0.7291666666666667</x:v>
+      </x:c>
+      <x:c r="I71" s="5" t="n">
+        <x:v>1.0208333333333333</x:v>
+      </x:c>
+      <x:c r="J71" s="6" t="n">
+        <x:v>56</x:v>
+      </x:c>
+      <x:c r="K71" s="6" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="L71" s="7" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M71" s="5" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="72">
+      <x:c r="A72" s="3" t="str">
+        <x:v>phase1_autumn_lumberjack</x:v>
+      </x:c>
+      <x:c r="B72" s="3" t="str">
+        <x:v>Chefe</x:v>
+      </x:c>
+      <x:c r="C72" s="11" t="str">
+        <x:v>Floresta Outono</x:v>
+      </x:c>
+      <x:c r="D72" s="4" t="str">
+        <x:v>Lenhador</x:v>
+      </x:c>
+      <x:c r="E72" s="3" t="str">
+        <x:v>vanguard</x:v>
+      </x:c>
+      <x:c r="F72" s="5" t="n">
+        <x:v>863.3333333333335</x:v>
+      </x:c>
+      <x:c r="G72" s="5" t="n">
+        <x:v>25.77916666666667</x:v>
+      </x:c>
+      <x:c r="H72" s="5" t="n">
+        <x:v>1.875</x:v>
+      </x:c>
+      <x:c r="I72" s="5" t="n">
+        <x:v>2.625</x:v>
+      </x:c>
+      <x:c r="J72" s="6" t="n">
+        <x:v>39.666666666666664</x:v>
+      </x:c>
+      <x:c r="K72" s="6" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="L72" s="7" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M72" s="5" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="73">
+      <x:c r="A73" s="3" t="str">
+        <x:v>phase1_spring_wolf</x:v>
+      </x:c>
+      <x:c r="B73" s="3" t="str">
+        <x:v>Comum</x:v>
+      </x:c>
+      <x:c r="C73" s="11" t="str">
+        <x:v>Floresta Primavera</x:v>
+      </x:c>
+      <x:c r="D73" s="4" t="str">
+        <x:v>Lobo Cinza</x:v>
+      </x:c>
+      <x:c r="E73" s="3" t="str">
+        <x:v>assassin</x:v>
+      </x:c>
+      <x:c r="F73" s="5" t="n">
+        <x:v>118.70833333333334</x:v>
+      </x:c>
+      <x:c r="G73" s="5" t="n">
+        <x:v>16.8125</x:v>
+      </x:c>
+      <x:c r="H73" s="5" t="n">
+        <x:v>0.6250000000000001</x:v>
+      </x:c>
+      <x:c r="I73" s="5" t="n">
+        <x:v>0.875</x:v>
+      </x:c>
+      <x:c r="J73" s="6" t="n">
+        <x:v>56</x:v>
+      </x:c>
+      <x:c r="K73" s="6" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="L73" s="7" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M73" s="5" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="74">
+      <x:c r="A74" s="3" t="str">
+        <x:v>phase1_spring_boar</x:v>
+      </x:c>
+      <x:c r="B74" s="3" t="str">
+        <x:v>Comum</x:v>
+      </x:c>
+      <x:c r="C74" s="11" t="str">
+        <x:v>Floresta Primavera</x:v>
+      </x:c>
+      <x:c r="D74" s="4" t="str">
+        <x:v>Javali</x:v>
+      </x:c>
+      <x:c r="E74" s="3" t="str">
+        <x:v>vanguard</x:v>
+      </x:c>
+      <x:c r="F74" s="5" t="n">
+        <x:v>215.83333333333337</x:v>
+      </x:c>
+      <x:c r="G74" s="5" t="n">
+        <x:v>15.691666666666668</x:v>
+      </x:c>
+      <x:c r="H74" s="5" t="n">
+        <x:v>1.4583333333333335</x:v>
+      </x:c>
+      <x:c r="I74" s="5" t="n">
+        <x:v>2.0416666666666665</x:v>
+      </x:c>
+      <x:c r="J74" s="6" t="n">
+        <x:v>44.33333333333333</x:v>
+      </x:c>
+      <x:c r="K74" s="6" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="L74" s="7" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M74" s="5" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="75">
+      <x:c r="A75" s="3" t="str">
+        <x:v>phase1_spring_hunter</x:v>
+      </x:c>
+      <x:c r="B75" s="3" t="str">
+        <x:v>Comum</x:v>
+      </x:c>
+      <x:c r="C75" s="11" t="str">
+        <x:v>Floresta Primavera</x:v>
+      </x:c>
+      <x:c r="D75" s="4" t="str">
+        <x:v>Caçador de Primavera</x:v>
+      </x:c>
+      <x:c r="E75" s="3" t="str">
+        <x:v>ranger</x:v>
+      </x:c>
+      <x:c r="F75" s="5" t="n">
+        <x:v>97.125</x:v>
+      </x:c>
+      <x:c r="G75" s="5" t="n">
+        <x:v>20.175</x:v>
+      </x:c>
+      <x:c r="H75" s="5" t="n">
+        <x:v>0.5208333333333334</x:v>
+      </x:c>
+      <x:c r="I75" s="5" t="n">
+        <x:v>0.7291666666666665</x:v>
+      </x:c>
+      <x:c r="J75" s="6" t="n">
+        <x:v>39.666666666666664</x:v>
+      </x:c>
+      <x:c r="K75" s="6" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="L75" s="7" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M75" s="5" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="76">
+      <x:c r="A76" s="3" t="str">
+        <x:v>phase1_spring_bear</x:v>
+      </x:c>
+      <x:c r="B76" s="3" t="str">
+        <x:v>Chefe</x:v>
+      </x:c>
+      <x:c r="C76" s="11" t="str">
+        <x:v>Floresta Primavera</x:v>
+      </x:c>
+      <x:c r="D76" s="4" t="str">
+        <x:v>Urso Pardo</x:v>
+      </x:c>
+      <x:c r="E76" s="3" t="str">
+        <x:v>vanguard</x:v>
+      </x:c>
+      <x:c r="F76" s="5" t="n">
+        <x:v>1036</x:v>
+      </x:c>
+      <x:c r="G76" s="5" t="n">
+        <x:v>25.77916666666667</x:v>
+      </x:c>
+      <x:c r="H76" s="5" t="n">
+        <x:v>2.3958333333333335</x:v>
+      </x:c>
+      <x:c r="I76" s="5" t="n">
+        <x:v>3.354166666666666</x:v>
+      </x:c>
+      <x:c r="J76" s="6" t="n">
+        <x:v>37.33333333333333</x:v>
+      </x:c>
+      <x:c r="K76" s="6" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="L76" s="7" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M76" s="5" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="77">
+      <x:c r="A77" s="3" t="str">
+        <x:v>phase1_summer_falcon</x:v>
+      </x:c>
+      <x:c r="B77" s="3" t="str">
+        <x:v>Comum</x:v>
+      </x:c>
+      <x:c r="C77" s="11" t="str">
+        <x:v>Floresta Verão</x:v>
+      </x:c>
+      <x:c r="D77" s="4" t="str">
+        <x:v>Falcão</x:v>
+      </x:c>
+      <x:c r="E77" s="3" t="str">
+        <x:v>assassin</x:v>
+      </x:c>
+      <x:c r="F77" s="5" t="n">
+        <x:v>86.33333333333334</x:v>
+      </x:c>
+      <x:c r="G77" s="5" t="n">
+        <x:v>15.691666666666668</x:v>
+      </x:c>
+      <x:c r="H77" s="5" t="n">
+        <x:v>0.41666666666666674</x:v>
+      </x:c>
+      <x:c r="I77" s="5" t="n">
+        <x:v>0.5833333333333333</x:v>
+      </x:c>
+      <x:c r="J77" s="6" t="n">
+        <x:v>63</x:v>
+      </x:c>
+      <x:c r="K77" s="6" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="L77" s="7" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M77" s="5" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="78">
+      <x:c r="A78" s="3" t="str">
+        <x:v>phase1_summer_raccoon</x:v>
+      </x:c>
+      <x:c r="B78" s="3" t="str">
+        <x:v>Comum</x:v>
+      </x:c>
+      <x:c r="C78" s="11" t="str">
+        <x:v>Floresta Verão</x:v>
+      </x:c>
+      <x:c r="D78" s="4" t="str">
+        <x:v>Guaxinim</x:v>
+      </x:c>
+      <x:c r="E78" s="3" t="str">
+        <x:v>vanguard</x:v>
+      </x:c>
+      <x:c r="F78" s="5" t="n">
+        <x:v>140.29166666666669</x:v>
+      </x:c>
+      <x:c r="G78" s="5" t="n">
+        <x:v>13.45</x:v>
+      </x:c>
+      <x:c r="H78" s="5" t="n">
+        <x:v>0.8333333333333335</x:v>
+      </x:c>
+      <x:c r="I78" s="5" t="n">
+        <x:v>1.1666666666666665</x:v>
+      </x:c>
+      <x:c r="J78" s="6" t="n">
+        <x:v>46.66666666666666</x:v>
+      </x:c>
+      <x:c r="K78" s="6" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="L78" s="7" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M78" s="5" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="79">
+      <x:c r="A79" s="3" t="str">
+        <x:v>phase1_summer_wolf</x:v>
+      </x:c>
+      <x:c r="B79" s="3" t="str">
+        <x:v>Comum</x:v>
+      </x:c>
+      <x:c r="C79" s="11" t="str">
+        <x:v>Floresta Verão</x:v>
+      </x:c>
+      <x:c r="D79" s="4" t="str">
+        <x:v>Lobo Marrom</x:v>
+      </x:c>
+      <x:c r="E79" s="3" t="str">
+        <x:v>assassin</x:v>
+      </x:c>
+      <x:c r="F79" s="5" t="n">
+        <x:v>118.70833333333334</x:v>
+      </x:c>
+      <x:c r="G79" s="5" t="n">
+        <x:v>17.933333333333334</x:v>
+      </x:c>
+      <x:c r="H79" s="5" t="n">
+        <x:v>0.6250000000000001</x:v>
+      </x:c>
+      <x:c r="I79" s="5" t="n">
+        <x:v>0.875</x:v>
+      </x:c>
+      <x:c r="J79" s="6" t="n">
+        <x:v>56</x:v>
+      </x:c>
+      <x:c r="K79" s="6" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="L79" s="7" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M79" s="5" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="80">
+      <x:c r="A80" s="3" t="str">
+        <x:v>phase1_summer_snake</x:v>
+      </x:c>
+      <x:c r="B80" s="3" t="str">
+        <x:v>Chefe</x:v>
+      </x:c>
+      <x:c r="C80" s="11" t="str">
+        <x:v>Floresta Verão</x:v>
+      </x:c>
+      <x:c r="D80" s="4" t="str">
+        <x:v>Serpente</x:v>
+      </x:c>
+      <x:c r="E80" s="3" t="str">
+        <x:v>assassin</x:v>
+      </x:c>
+      <x:c r="F80" s="5" t="n">
+        <x:v>777</x:v>
+      </x:c>
+      <x:c r="G80" s="5" t="n">
+        <x:v>28.020833333333336</x:v>
+      </x:c>
+      <x:c r="H80" s="5" t="n">
+        <x:v>1.354166666666667</x:v>
+      </x:c>
+      <x:c r="I80" s="5" t="n">
+        <x:v>1.895833333333333</x:v>
+      </x:c>
+      <x:c r="J80" s="6" t="n">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="K80" s="6" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="L80" s="7" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M80" s="5" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="F2:M64">
     <x:cfRule type="expression" dxfId="0" priority="1">
@@ -3076,7 +3732,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd2045322040743b9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0afbca2b5a3f4cea"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3149,7 +3805,7 @@
     </x:row>
     <x:row r="9" ht="32" customHeight="1">
       <x:c r="B9" s="24" t="str">
-        <x:v>Colunas cinza</x:v>
+        <x:v>id, tipo, bioma e classe são referências. Mantenha os IDs, cabeçalhos e todas as 79 linhas.</x:v>
       </x:c>
       <x:c r="C9" s="25" t="str">
         <x:v>id, tipo, bioma e classe são referências. Mantenha os IDs, cabeçalhos e todas as 63 linhas.</x:v>

</xml_diff>